<commit_message>
update carbon major iso mapping
</commit_message>
<xml_diff>
--- a/data/packaged/carbon_major_iso_mapping.xlsx
+++ b/data/packaged/carbon_major_iso_mapping.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iiasahub-my.sharepoint.com/personal/gidden_iiasa_ac_at/Documents/work/iiasa/papers/2024-cstorage/2024_gidden_cstorage/data/packaged/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pnnl-my.sharepoint.com/personal/matthew_gidden_pnnl_gov/Documents/Documents/work/papers/2024_gidden_cstorage/data/packaged/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_23F921EDCC530C0F1D2D4CDBEDC845E86B189EB8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B1DE071-8A8F-4898-BEB5-BC8974ECC482}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_23F921EDCC530C0F1D2D4CDBEDC845E86B189EB8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6A536A2-D8B6-2E45-819A-91A82AEEB306}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30480" yWindow="2560" windowWidth="23260" windowHeight="12580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="v1" sheetId="1" r:id="rId1"/>
+    <sheet name="v2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="302">
   <si>
     <t>name</t>
   </si>
@@ -653,13 +654,286 @@
   </si>
   <si>
     <t>Argentina</t>
+  </si>
+  <si>
+    <t>Former Soviet Union (1900-1991)</t>
+  </si>
+  <si>
+    <t>FSU</t>
+  </si>
+  <si>
+    <t>China (Coal, 1945-2004)</t>
+  </si>
+  <si>
+    <t>National Iranian Oil Company</t>
+  </si>
+  <si>
+    <t>Iran</t>
+  </si>
+  <si>
+    <t>UK</t>
+  </si>
+  <si>
+    <t>Poland (Coal, 1913–2001)</t>
+  </si>
+  <si>
+    <t>CHN Energy</t>
+  </si>
+  <si>
+    <t>British Coal Corporation (1947-1994)</t>
+  </si>
+  <si>
+    <t>Peabody Energy</t>
+  </si>
+  <si>
+    <t>Venezuela</t>
+  </si>
+  <si>
+    <t>Jinneng Group</t>
+  </si>
+  <si>
+    <t>Shandong Energy</t>
+  </si>
+  <si>
+    <t>Czechoslovakia (Coal, 1938-1992)</t>
+  </si>
+  <si>
+    <t>China National Coal Group</t>
+  </si>
+  <si>
+    <t>Shanxi Coking Coal Group</t>
+  </si>
+  <si>
+    <t>Rio Tinto (1959-2018)</t>
+  </si>
+  <si>
+    <t>Shaanxi Coal and Chemical Industry Group</t>
+  </si>
+  <si>
+    <t>ONGC</t>
+  </si>
+  <si>
+    <t>SUEK</t>
+  </si>
+  <si>
+    <t>North Korea</t>
+  </si>
+  <si>
+    <t>PRK</t>
+  </si>
+  <si>
+    <t>Henan Energy and Chemical Industry Group</t>
+  </si>
+  <si>
+    <t>Samruk-Kazyna</t>
+  </si>
+  <si>
+    <t>China Huaneng Group</t>
+  </si>
+  <si>
+    <t>State Power Investment Corporation</t>
+  </si>
+  <si>
+    <t>Luan Chemical Group</t>
+  </si>
+  <si>
+    <t>Jizhong Energy Resources</t>
+  </si>
+  <si>
+    <t>Huaihe Energy Holding Group</t>
+  </si>
+  <si>
+    <t>Huayang New Material Technology Group</t>
+  </si>
+  <si>
+    <t>Liaoning Energy Industry Holding Group</t>
+  </si>
+  <si>
+    <t>Ukrainian Ministry of Energy (Coal, 1992-2012)</t>
+  </si>
+  <si>
+    <t>Kuzbassrazrezugol</t>
+  </si>
+  <si>
+    <t>Cyprus AMAX Minerals (1969-1998)</t>
+  </si>
+  <si>
+    <t>Kailuan Group</t>
+  </si>
+  <si>
+    <t>Polska Grupa Gornicza (PGG)</t>
+  </si>
+  <si>
+    <t>Heilongjiang Longmay Mining Holding Group</t>
+  </si>
+  <si>
+    <t>Inner Mongolia Yitai Group</t>
+  </si>
+  <si>
+    <t>AlamTri Resources</t>
+  </si>
+  <si>
+    <t>Mitsubishi Corporation</t>
+  </si>
+  <si>
+    <t>Inner Mongolia Dian Tou Energy</t>
+  </si>
+  <si>
+    <t>Tatneft</t>
+  </si>
+  <si>
+    <t>Eurasian Resources Group</t>
+  </si>
+  <si>
+    <t>Luxembourg</t>
+  </si>
+  <si>
+    <t>LUX</t>
+  </si>
+  <si>
+    <t>China Pingmei Shenma Energy and Chemicals Group</t>
+  </si>
+  <si>
+    <t>NACCO Industries</t>
+  </si>
+  <si>
+    <t>INPEX</t>
+  </si>
+  <si>
+    <t>Syria</t>
+  </si>
+  <si>
+    <t>Inner Mongolia Huineng Coal and Electricity Group</t>
+  </si>
+  <si>
+    <t>Huadian Coal Industry Group</t>
+  </si>
+  <si>
+    <t>Huaibei Mining Group</t>
+  </si>
+  <si>
+    <t>Cloud Peak (2009-2019)</t>
+  </si>
+  <si>
+    <t>EVRAZ</t>
+  </si>
+  <si>
+    <t>PGE Group</t>
+  </si>
+  <si>
+    <t>DTEK</t>
+  </si>
+  <si>
+    <t>Mechel</t>
+  </si>
+  <si>
+    <t>Inner Mongolia Yidong Resources Group</t>
+  </si>
+  <si>
+    <t>Guizhou Panjiang Coal Power Group</t>
+  </si>
+  <si>
+    <t>Xuzhou Mining Group</t>
+  </si>
+  <si>
+    <t>Inner Mongolia Mengtai Group</t>
+  </si>
+  <si>
+    <t>OMV</t>
+  </si>
+  <si>
+    <t>Huating Coal Industry Group</t>
+  </si>
+  <si>
+    <t>UK Coal (1995-2015)</t>
+  </si>
+  <si>
+    <t>SDS Coal</t>
+  </si>
+  <si>
+    <t>En+ Group</t>
+  </si>
+  <si>
+    <t>JSW</t>
+  </si>
+  <si>
+    <t>Mubadala</t>
+  </si>
+  <si>
+    <t>Severstal</t>
+  </si>
+  <si>
+    <t>Antero Resources</t>
+  </si>
+  <si>
+    <t>Novaya Gornaya</t>
+  </si>
+  <si>
+    <t>Metinvest</t>
+  </si>
+  <si>
+    <t>ARC Resources</t>
+  </si>
+  <si>
+    <t>Russian Coal</t>
+  </si>
+  <si>
+    <t>Kazakhmys Holding Group</t>
+  </si>
+  <si>
+    <t>UltraTech Cement</t>
+  </si>
+  <si>
+    <t>ELSI</t>
+  </si>
+  <si>
+    <t>ArcelorMittal</t>
+  </si>
+  <si>
+    <t>Kuzbasskaya Toplivnaya</t>
+  </si>
+  <si>
+    <t>Xinjiang Tianchi Energy</t>
+  </si>
+  <si>
+    <t>Adani Group</t>
+  </si>
+  <si>
+    <t>Severoceske doly</t>
+  </si>
+  <si>
+    <t>Stroyservis</t>
+  </si>
+  <si>
+    <t>LW Bogdanka</t>
+  </si>
+  <si>
+    <t>OKD</t>
+  </si>
+  <si>
+    <t>Vale (2007-2022)</t>
+  </si>
+  <si>
+    <t>Sev.en Group</t>
+  </si>
+  <si>
+    <t>Poludniowy Koncern Weglowy</t>
+  </si>
+  <si>
+    <t>Sokolovska uhelna</t>
+  </si>
+  <si>
+    <t>TALTEK</t>
+  </si>
+  <si>
+    <t>Elgaugol</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -671,6 +945,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -711,11 +992,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -733,10 +1015,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -774,9 +1060,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -809,26 +1095,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -861,26 +1130,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1055,14 +1307,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C122"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1073,7 +1325,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1084,7 +1336,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1095,7 +1347,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1106,7 +1358,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1117,7 +1369,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1128,7 +1380,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1139,7 +1391,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1150,7 +1402,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1161,7 +1413,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1172,7 +1424,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1183,7 +1435,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1194,7 +1446,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -1205,7 +1457,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -1216,7 +1468,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1227,7 +1479,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1238,7 +1490,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -1249,7 +1501,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -1260,7 +1512,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -1271,7 +1523,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1282,7 +1534,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -1293,7 +1545,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -1304,7 +1556,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -1315,7 +1567,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -1326,7 +1578,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -1337,7 +1589,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -1348,7 +1600,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -1359,7 +1611,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -1370,7 +1622,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -1381,7 +1633,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>31</v>
       </c>
@@ -1392,7 +1644,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1403,7 +1655,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -1414,7 +1666,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -1425,7 +1677,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1436,7 +1688,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>36</v>
       </c>
@@ -1447,7 +1699,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -1458,7 +1710,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -1469,7 +1721,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -1480,7 +1732,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -1491,7 +1743,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -1502,7 +1754,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>42</v>
       </c>
@@ -1513,7 +1765,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>43</v>
       </c>
@@ -1524,7 +1776,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>44</v>
       </c>
@@ -1535,7 +1787,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>45</v>
       </c>
@@ -1546,7 +1798,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -1557,7 +1809,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>47</v>
       </c>
@@ -1568,7 +1820,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -1579,7 +1831,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>49</v>
       </c>
@@ -1590,7 +1842,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>50</v>
       </c>
@@ -1601,7 +1853,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>51</v>
       </c>
@@ -1612,7 +1864,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>52</v>
       </c>
@@ -1623,7 +1875,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>53</v>
       </c>
@@ -1634,7 +1886,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>54</v>
       </c>
@@ -1645,7 +1897,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>55</v>
       </c>
@@ -1656,7 +1908,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>56</v>
       </c>
@@ -1667,7 +1919,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>57</v>
       </c>
@@ -1678,7 +1930,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>58</v>
       </c>
@@ -1689,7 +1941,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>59</v>
       </c>
@@ -1700,7 +1952,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>60</v>
       </c>
@@ -1711,7 +1963,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>61</v>
       </c>
@@ -1722,7 +1974,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>62</v>
       </c>
@@ -1733,7 +1985,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>63</v>
       </c>
@@ -1744,7 +1996,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>64</v>
       </c>
@@ -1755,7 +2007,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>65</v>
       </c>
@@ -1766,7 +2018,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>66</v>
       </c>
@@ -1777,7 +2029,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>67</v>
       </c>
@@ -1788,7 +2040,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>68</v>
       </c>
@@ -1799,7 +2051,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>69</v>
       </c>
@@ -1810,7 +2062,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>70</v>
       </c>
@@ -1821,7 +2073,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>71</v>
       </c>
@@ -1832,7 +2084,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>72</v>
       </c>
@@ -1843,7 +2095,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>73</v>
       </c>
@@ -1854,7 +2106,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>74</v>
       </c>
@@ -1865,7 +2117,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>75</v>
       </c>
@@ -1876,7 +2128,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>76</v>
       </c>
@@ -1887,7 +2139,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>77</v>
       </c>
@@ -1898,7 +2150,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>78</v>
       </c>
@@ -1909,7 +2161,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>79</v>
       </c>
@@ -1920,7 +2172,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>80</v>
       </c>
@@ -1931,7 +2183,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>81</v>
       </c>
@@ -1942,7 +2194,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>82</v>
       </c>
@@ -1953,7 +2205,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -1964,7 +2216,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>84</v>
       </c>
@@ -1975,7 +2227,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>85</v>
       </c>
@@ -1986,7 +2238,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>86</v>
       </c>
@@ -1997,7 +2249,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>87</v>
       </c>
@@ -2008,7 +2260,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>88</v>
       </c>
@@ -2019,7 +2271,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>89</v>
       </c>
@@ -2030,7 +2282,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>90</v>
       </c>
@@ -2041,7 +2293,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>91</v>
       </c>
@@ -2052,7 +2304,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>92</v>
       </c>
@@ -2063,7 +2315,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>93</v>
       </c>
@@ -2074,7 +2326,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>94</v>
       </c>
@@ -2085,7 +2337,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>95</v>
       </c>
@@ -2096,7 +2348,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>96</v>
       </c>
@@ -2107,7 +2359,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>97</v>
       </c>
@@ -2118,7 +2370,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>98</v>
       </c>
@@ -2129,7 +2381,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>99</v>
       </c>
@@ -2140,7 +2392,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>100</v>
       </c>
@@ -2151,7 +2403,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>101</v>
       </c>
@@ -2162,7 +2414,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>102</v>
       </c>
@@ -2173,7 +2425,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>103</v>
       </c>
@@ -2184,7 +2436,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>104</v>
       </c>
@@ -2195,7 +2447,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>105</v>
       </c>
@@ -2206,7 +2458,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>106</v>
       </c>
@@ -2217,7 +2469,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>107</v>
       </c>
@@ -2228,7 +2480,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>108</v>
       </c>
@@ -2239,7 +2491,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>109</v>
       </c>
@@ -2250,7 +2502,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>110</v>
       </c>
@@ -2261,7 +2513,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>111</v>
       </c>
@@ -2272,7 +2524,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>112</v>
       </c>
@@ -2283,7 +2535,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>113</v>
       </c>
@@ -2294,7 +2546,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>114</v>
       </c>
@@ -2305,7 +2557,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>115</v>
       </c>
@@ -2316,7 +2568,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>116</v>
       </c>
@@ -2327,7 +2579,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>117</v>
       </c>
@@ -2338,7 +2590,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>118</v>
       </c>
@@ -2349,7 +2601,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>119</v>
       </c>
@@ -2360,7 +2612,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>120</v>
       </c>
@@ -2371,7 +2623,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>121</v>
       </c>
@@ -2382,7 +2634,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>122</v>
       </c>
@@ -2393,7 +2645,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>123</v>
       </c>
@@ -2402,6 +2654,2007 @@
       </c>
       <c r="C122" t="s">
         <v>210</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AD6538B-7316-CD4D-B11B-4CC10F718BBB}">
+  <dimension ref="A1:C181"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A105" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A107" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A108" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A109" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A110" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A111" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A112" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A113" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A114" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A115" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A116" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A117" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A118" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A119" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A120" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A121" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A122" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A123" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A124" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A125" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A126" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A127" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A128" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A129" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A130" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A131" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A132" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A133" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A134" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A135" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A136" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A137" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A138" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A139" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A140" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A141" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A142" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A143" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A144" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A145" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A146" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A147" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A148" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A149" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A150" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A151" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A152" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A153" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A154" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A155" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A156" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A157" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A158" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A159" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A160" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A161" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A162" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A163" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A164" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A165" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A166" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A167" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A168" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A169" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A170" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A171" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A172" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A173" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A174" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A175" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B175" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A176" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A177" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A178" t="s">
+        <v>113</v>
+      </c>
+      <c r="B178" t="s">
+        <v>216</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A179" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A180" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A181" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>